<commit_message>
update zy1001 report github fields
</commit_message>
<xml_diff>
--- a/result_data/zy1001.xlsx
+++ b/result_data/zy1001.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据表" sheetId="1" r:id="Re9cf21cd1f5d4d06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据表" sheetId="1" r:id="Rb80482b3902744ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -213,6 +213,12 @@
       <x:c r="G1" t="str">
         <x:v>不满意原因</x:v>
       </x:c>
+      <x:c r="H1" t="str">
+        <x:v>远端Github地址</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>分支文件夹</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
@@ -240,6 +246,12 @@
       <x:c r="G2" t="str">
         <x:v>产物不满意：前后端构建均失败，项目无法按说明运行。</x:v>
       </x:c>
+      <x:c r="H2" t="str">
+        <x:v>https://github.com/lizyyy/solo/tree/pro/zy1001</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>pro/zy1001</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refine zy1001 report reason
</commit_message>
<xml_diff>
--- a/result_data/zy1001.xlsx
+++ b/result_data/zy1001.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据表" sheetId="1" r:id="Rb80482b3902744ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据表" sheetId="1" r:id="R8c449ab11edb486b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -244,7 +244,7 @@
         <x:v>不满意</x:v>
       </x:c>
       <x:c r="G2" t="str">
-        <x:v>产物不满意：前后端构建均失败，项目无法按说明运行。</x:v>
+        <x:v>产物不满意：生产打包命令失败，README前端访问端口写成3000但实际为3002。</x:v>
       </x:c>
       <x:c r="H2" t="str">
         <x:v>https://github.com/lizyyy/solo/tree/pro/zy1001</x:v>

</xml_diff>